<commit_message>
Regenerate public TID catalog: add Seek Position (103), Jog Turn, Scratch, etc.
Rebuilt TID_catalog_public.xlsx from the updated master. Adds own-authored
descriptions for Seek Position (103), Jog Turn (120), Scratch (121), Jog Touch
On (2187), Scratch Control On (2288), Preview-player seek (211); 103 now marked
Proven (hardware-tested) - drives the swing-skip Dial seek.
</commit_message>
<xml_diff>
--- a/release_GideonSTEM-Maschine/TID_catalog_public.xlsx
+++ b/release_GideonSTEM-Maschine/TID_catalog_public.xlsx
@@ -939,33 +939,37 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="4" t="n">
         <v>103</v>
       </c>
-      <c r="B13" s="3" t="inlineStr"/>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Seek Position (relative; scrubs the playhead through the track - responsive, no quantize)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
         <is>
           <t>Button, Knob, LED</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Dec, Direct, Inc, Output</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" s="4" t="inlineStr">
         <is>
           <t>-1, 0, 1</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="G13" s="3" t="inlineStr">
-        <is>
-          <t>Documented</t>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
+        <is>
+          <t>Proven (hardware-tested)</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1039,11 @@
       <c r="A16" s="3" t="n">
         <v>120</v>
       </c>
-      <c r="B16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Jog Turn (centered float; jog-wheel nudge / pitch-bend)</t>
+        </is>
+      </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Button</t>
@@ -1361,7 +1369,11 @@
       <c r="A26" s="3" t="n">
         <v>211</v>
       </c>
-      <c r="B26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Seek Position - Preview Player (relative)</t>
+        </is>
+      </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
           <t>Encoder</t>
@@ -9204,7 +9216,11 @@
       <c r="A271" t="n">
         <v>2187</v>
       </c>
-      <c r="B271" t="inlineStr"/>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Jog Touch On (jog capacitive touch)</t>
+        </is>
+      </c>
       <c r="C271" t="inlineStr">
         <is>
           <t>Button, LED</t>
@@ -9518,7 +9534,11 @@
       <c r="A281" s="3" t="n">
         <v>2288</v>
       </c>
-      <c r="B281" s="3" t="inlineStr"/>
+      <c r="B281" s="3" t="inlineStr">
+        <is>
+          <t>Scratch Control On</t>
+        </is>
+      </c>
       <c r="C281" s="3" t="inlineStr">
         <is>
           <t>Button, LED</t>

</xml_diff>